<commit_message>
TE-11:Table & TestCases State Transition
</commit_message>
<xml_diff>
--- a/postman/BVA/TE8_BVA_TestCases.xlsx
+++ b/postman/BVA/TE8_BVA_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lala/Documents/GitHub/KCPM-WEDNESDAY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lala/Documents/GitHub/KCPM-WEDNESDAY/postman/BVA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33CB10D5-0A10-CF48-838B-48BDD8BCE909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9FB419-C485-4241-A1D3-5AD51FD51B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9560" yWindow="760" windowWidth="20680" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9560" yWindow="760" windowWidth="20680" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Phân tích BVA" sheetId="1" r:id="rId1"/>
@@ -1383,7 +1383,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1503,11 +1503,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1536,6 +1556,45 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1548,62 +1607,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1910,486 +1954,486 @@
   <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.1640625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17" style="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5" style="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.1640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5" style="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.1640625" style="18"/>
+    <col min="1" max="1" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="10.1640625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="14" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
-      <c r="B4" s="23" t="s">
+      <c r="A4" s="24"/>
+      <c r="B4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="15" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23" t="s">
+      <c r="A5" s="24"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="15" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23" t="s">
+      <c r="A6" s="24"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="15" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24" t="s">
+      <c r="A7" s="25"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="15" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="14" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="23" t="s">
+      <c r="A9" s="24"/>
+      <c r="B9" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="15" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24" t="s">
+      <c r="A10" s="25"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="16" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="F11" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="G11" s="15" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="B12" s="23" t="s">
+      <c r="A12" s="24"/>
+      <c r="B12" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="G12" s="15" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23" t="s">
+      <c r="A13" s="24"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="15" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23" t="s">
+      <c r="A14" s="24"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="15" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24" t="s">
+      <c r="A15" s="25"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="G15" s="24" t="s">
+      <c r="G15" s="16" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G17" s="30" t="s">
+      <c r="G17" s="20" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="14" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23" t="s">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="23" t="s">
+      <c r="G19" s="15" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23" t="s">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="23" t="s">
+      <c r="G20" s="15" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="28" t="s">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G21" s="15" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="29" t="s">
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="16" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="27" t="s">
+      <c r="F23" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G23" s="23" t="s">
+      <c r="G23" s="15" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23" t="s">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="E24" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="G24" s="23" t="s">
+      <c r="G24" s="15" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="28" t="s">
+      <c r="A25" s="15"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" s="15" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="28" t="s">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="G26" s="23" t="s">
+      <c r="G26" s="15" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="24"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="29" t="s">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G27" s="24" t="s">
+      <c r="G27" s="16" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2421,31 +2465,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="11" t="s">
         <v>36</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="23" t="s">
         <v>59</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -2454,35 +2498,35 @@
       <c r="C3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="23" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
+      <c r="A4" s="24"/>
       <c r="B4" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="11"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="24"/>
     </row>
     <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
+      <c r="A5" s="25"/>
       <c r="B5" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="12"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="25"/>
     </row>
     <row r="6" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="23" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -2491,35 +2535,35 @@
       <c r="C6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="23" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="11"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="11"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="8" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12"/>
+      <c r="A8" s="25"/>
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="11"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="24"/>
     </row>
     <row r="9" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="23" t="s">
         <v>61</v>
       </c>
       <c r="B9" s="7" t="s">
@@ -2528,33 +2572,33 @@
       <c r="C9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="11"/>
+      <c r="E9" s="24"/>
     </row>
     <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
+      <c r="A10" s="24"/>
       <c r="B10" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="11"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="24"/>
     </row>
     <row r="11" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
+      <c r="A11" s="25"/>
       <c r="B11" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="11"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="24"/>
     </row>
     <row r="12" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -2563,33 +2607,33 @@
       <c r="C12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="E12" s="11"/>
+      <c r="E12" s="24"/>
     </row>
     <row r="13" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="11"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="24"/>
     </row>
     <row r="14" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
+      <c r="A14" s="25"/>
       <c r="B14" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C14" s="6"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="11"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="24"/>
     </row>
     <row r="15" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="23" t="s">
         <v>63</v>
       </c>
       <c r="B15" s="7" t="s">
@@ -2598,33 +2642,33 @@
       <c r="C15" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="24"/>
     </row>
     <row r="16" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="11"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="24"/>
     </row>
     <row r="17" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
+      <c r="A17" s="25"/>
       <c r="B17" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="6"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="11"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="24"/>
     </row>
     <row r="18" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="23" t="s">
         <v>64</v>
       </c>
       <c r="B18" s="7" t="s">
@@ -2633,35 +2677,35 @@
       <c r="C18" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="24" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="8" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="11"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="24"/>
     </row>
     <row r="20" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
+      <c r="A20" s="25"/>
       <c r="B20" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C20" s="6"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="11"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="24"/>
     </row>
     <row r="21" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="23" t="s">
         <v>65</v>
       </c>
       <c r="B21" s="7" t="s">
@@ -2670,33 +2714,33 @@
       <c r="C21" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="24"/>
     </row>
     <row r="22" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="8" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="11"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="24"/>
     </row>
     <row r="23" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12"/>
+      <c r="A23" s="25"/>
       <c r="B23" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C23" s="6"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="11"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="24"/>
     </row>
     <row r="24" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="23" t="s">
         <v>66</v>
       </c>
       <c r="B24" s="7" t="s">
@@ -2705,35 +2749,35 @@
       <c r="C24" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="24" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="11"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="26" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="12"/>
+      <c r="A26" s="25"/>
       <c r="B26" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C26" s="6"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="11"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="24"/>
     </row>
     <row r="27" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="23" t="s">
         <v>67</v>
       </c>
       <c r="B27" s="7" t="s">
@@ -2742,33 +2786,33 @@
       <c r="C27" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="E27" s="11"/>
+      <c r="E27" s="24"/>
     </row>
     <row r="28" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="11"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="24"/>
     </row>
     <row r="29" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="12"/>
+      <c r="A29" s="25"/>
       <c r="B29" s="9" t="s">
         <v>55</v>
       </c>
       <c r="C29" s="6"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="11"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="24"/>
     </row>
     <row r="30" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B30" s="7" t="s">
@@ -2777,33 +2821,33 @@
       <c r="C30" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="E30" s="11"/>
+      <c r="E30" s="24"/>
     </row>
     <row r="31" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="11"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="24"/>
     </row>
     <row r="32" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="12"/>
+      <c r="A32" s="25"/>
       <c r="B32" s="9" t="s">
         <v>56</v>
       </c>
       <c r="C32" s="6"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="11"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="24"/>
     </row>
     <row r="33" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="23" t="s">
         <v>69</v>
       </c>
       <c r="B33" s="7" t="s">
@@ -2812,55 +2856,55 @@
       <c r="C33" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="11"/>
+      <c r="E33" s="24"/>
     </row>
     <row r="34" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
+      <c r="A34" s="24"/>
       <c r="B34" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="11"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="24"/>
     </row>
     <row r="35" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="12"/>
+      <c r="A35" s="25"/>
       <c r="B35" s="9" t="s">
         <v>57</v>
       </c>
       <c r="C35" s="6"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="12"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="25"/>
     </row>
     <row r="36" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="25" t="s">
+      <c r="A36" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="30"/>
     </row>
     <row r="37" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="19" t="s">
+      <c r="A37" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="19" t="s">
+      <c r="B37" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="C37" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="11" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="28" t="s">
         <v>130</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -2869,26 +2913,26 @@
       <c r="C38" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="E38" s="31" t="s">
+      <c r="E38" s="28" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="31"/>
-      <c r="B39" s="32" t="s">
+      <c r="A39" s="28"/>
+      <c r="B39" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D39" s="15"/>
-      <c r="E39" s="31"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="28"/>
     </row>
     <row r="40" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="28" t="s">
         <v>131</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -2897,26 +2941,26 @@
       <c r="C40" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="26" t="s">
         <v>161</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="28" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="31"/>
-      <c r="B41" s="32" t="s">
+      <c r="A41" s="28"/>
+      <c r="B41" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D41" s="15"/>
-      <c r="E41" s="31"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="31" t="s">
+      <c r="A42" s="28" t="s">
         <v>132</v>
       </c>
       <c r="B42" s="4" t="s">
@@ -2925,24 +2969,24 @@
       <c r="C42" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="E42" s="31"/>
+      <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="31"/>
-      <c r="B43" s="32" t="s">
+      <c r="A43" s="28"/>
+      <c r="B43" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D43" s="15"/>
-      <c r="E43" s="31"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="28"/>
     </row>
     <row r="44" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="31" t="s">
+      <c r="A44" s="28" t="s">
         <v>133</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -2951,24 +2995,24 @@
       <c r="C44" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="E44" s="31"/>
+      <c r="E44" s="28"/>
     </row>
     <row r="45" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="31"/>
-      <c r="B45" s="32" t="s">
+      <c r="A45" s="28"/>
+      <c r="B45" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D45" s="15"/>
-      <c r="E45" s="31"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
     </row>
     <row r="46" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="31" t="s">
+      <c r="A46" s="28" t="s">
         <v>134</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -2977,24 +3021,24 @@
       <c r="C46" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="E46" s="31"/>
+      <c r="E46" s="28"/>
     </row>
     <row r="47" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="31"/>
-      <c r="B47" s="32" t="s">
+      <c r="A47" s="28"/>
+      <c r="B47" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D47" s="15"/>
-      <c r="E47" s="31"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="28"/>
     </row>
     <row r="48" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="31" t="s">
+      <c r="A48" s="28" t="s">
         <v>135</v>
       </c>
       <c r="B48" s="4" t="s">
@@ -3003,26 +3047,26 @@
       <c r="C48" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="E48" s="31" t="s">
+      <c r="E48" s="28" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="31"/>
-      <c r="B49" s="32" t="s">
+      <c r="A49" s="28"/>
+      <c r="B49" s="21" t="s">
         <v>167</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D49" s="15"/>
-      <c r="E49" s="31"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="28"/>
     </row>
     <row r="50" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="31" t="s">
+      <c r="A50" s="28" t="s">
         <v>136</v>
       </c>
       <c r="B50" s="4" t="s">
@@ -3031,24 +3075,24 @@
       <c r="C50" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="D50" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="E50" s="31"/>
+      <c r="E50" s="28"/>
     </row>
     <row r="51" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="31"/>
-      <c r="B51" s="32" t="s">
+      <c r="A51" s="28"/>
+      <c r="B51" s="21" t="s">
         <v>168</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D51" s="15"/>
-      <c r="E51" s="31"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="28"/>
     </row>
     <row r="52" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="31" t="s">
+      <c r="A52" s="28" t="s">
         <v>137</v>
       </c>
       <c r="B52" s="4" t="s">
@@ -3057,24 +3101,24 @@
       <c r="C52" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="E52" s="31"/>
+      <c r="E52" s="28"/>
     </row>
     <row r="53" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="31"/>
-      <c r="B53" s="32" t="s">
+      <c r="A53" s="28"/>
+      <c r="B53" s="21" t="s">
         <v>169</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D53" s="15"/>
-      <c r="E53" s="31"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="28"/>
     </row>
     <row r="54" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="31" t="s">
+      <c r="A54" s="28" t="s">
         <v>138</v>
       </c>
       <c r="B54" s="4" t="s">
@@ -3083,32 +3127,46 @@
       <c r="C54" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D54" s="13" t="s">
+      <c r="D54" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="E54" s="31"/>
+      <c r="E54" s="28"/>
     </row>
     <row r="55" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="31"/>
-      <c r="B55" s="32" t="s">
+      <c r="A55" s="28"/>
+      <c r="B55" s="21" t="s">
         <v>170</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D55" s="15"/>
-      <c r="E55" s="31"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E6:E17"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E40:E47"/>
-    <mergeCell ref="E48:E55"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A50:A51"/>
     <mergeCell ref="A52:A53"/>
     <mergeCell ref="A54:A55"/>
@@ -3124,32 +3182,18 @@
     <mergeCell ref="D42:D43"/>
     <mergeCell ref="D44:D45"/>
     <mergeCell ref="D46:D47"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="D15:D17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E6:E17"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E40:E47"/>
+    <mergeCell ref="E48:E55"/>
     <mergeCell ref="E18:E23"/>
     <mergeCell ref="E24:E35"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="D27:D29"/>
     <mergeCell ref="D30:D32"/>
     <mergeCell ref="D33:D35"/>
-    <mergeCell ref="E3:E5"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>